<commit_message>
docs: actualizar descripciones explicitas en linea base y final
</commit_message>
<xml_diff>
--- a/Laboratorio_2_Evidencias.xlsx
+++ b/Laboratorio_2_Evidencias.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin fallo (ejecucion limpia inicial)</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Estado inicial correcto</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>F401 `os` imported but unused</t>
+          <t>F401 os imported but unused</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sin fallo (verificacion final limpia)</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Todos los controles remediados</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">

</xml_diff>